<commit_message>
docs: add syslog security documentation and acceptance scenarios
</commit_message>
<xml_diff>
--- a/docs/security/03_Akceptacni_testy_se_screenshoty.xlsx
+++ b/docs/security/03_Akceptacni_testy_se_screenshoty.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Akceptační testy" sheetId="1" r:id="R1ef63057c9a1481f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Souhrn" sheetId="2" r:id="Re43cbf0779f948cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="3" r:id="Re40dcc4a3fcd4a0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Akceptační testy" sheetId="1" r:id="Radea325c32324bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Souhrn" sheetId="2" r:id="R9f31c8b78c2341c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="3" r:id="R9ebd90119d274032"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="10">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -71,6 +71,15 @@
       <x:color rgb="FF7F3300"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
   <x:fills count="7">
     <x:fill>
@@ -112,7 +121,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="62">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -236,11 +245,16 @@
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="6">
+  <x:dxfs count="9">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -306,6 +320,27 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE7E6E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
@@ -322,13 +357,13 @@
     <xdr:ext cx="10477500" cy="5130297"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="963fe2a3-7780-47fe-ab13-82e272a0634d"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6e3005d85f7e4595"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbd0edbaa31c5428d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -349,13 +384,13 @@
     <xdr:ext cx="9486900" cy="2924175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="99cae602-4e39-4914-af9c-dce1075bbd13"/>
+        <xdr:cNvPr id="2" name="/xl/media/image2.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9e4ab622dcf740d5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R472ff8a4890d48cf"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -376,13 +411,13 @@
     <xdr:ext cx="9486900" cy="4286250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="f6780716-94eb-4995-add5-fcd23936edf4"/>
+        <xdr:cNvPr id="3" name="/xl/media/image3.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1b39ada731994cf8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re7d4be4be91d4c07"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -403,13 +438,13 @@
     <xdr:ext cx="9486900" cy="2705100"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="2ef91615-af14-4485-b073-5e4838960d57"/>
+        <xdr:cNvPr id="4" name="/xl/media/image4.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7ec208a7a21842a0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Reb6e085698cc459c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -430,13 +465,13 @@
     <xdr:ext cx="9486900" cy="4676775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="f6cf4d52-4ad3-45e0-b1c9-e28de7d2e857"/>
+        <xdr:cNvPr id="5" name="/xl/media/image5.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3b3cdae5e4a846dd"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3c4aa7e63f2447da"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -457,13 +492,13 @@
     <xdr:ext cx="10477500" cy="4286250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="61d92c6f-fc51-48a8-9287-22b40dbc102d"/>
+        <xdr:cNvPr id="6" name="/xl/media/image6.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re8a8a683b0834d59"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R76700be50b334f67"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -484,13 +519,13 @@
     <xdr:ext cx="10439400" cy="4019550"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="edfba1d9-cf32-4116-9c8d-d83c2ad6a7dd"/>
+        <xdr:cNvPr id="7" name="/xl/media/image7.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0bf4a3654bbc4a6c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0899012ca1c341e9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -511,13 +546,13 @@
     <xdr:ext cx="5229225" cy="3743325"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="54b985da-2c46-4342-b241-198f8665cc07"/>
+        <xdr:cNvPr id="8" name="/xl/media/image8.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re4c0ef66bb10432b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rae64b14f5b134e04"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -538,13 +573,13 @@
     <xdr:ext cx="10439400" cy="4676775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="9c47e62e-19b3-4093-91f2-bfba6ff905d8"/>
+        <xdr:cNvPr id="9" name="/xl/media/image9.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R57c3694f47bc40de"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2d7e2c3cd42449e3"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -565,13 +600,13 @@
     <xdr:ext cx="10439400" cy="4895850"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="5467c966-fb7b-4b02-b805-8f8af4a49cbf"/>
+        <xdr:cNvPr id="10" name="/xl/media/image10.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R69d19f52c3c442e4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc5d6710d31af4fae"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -592,13 +627,13 @@
     <xdr:ext cx="10439400" cy="2009775"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="9899835b-ea83-47a0-9ba5-b2b09c3645fb"/>
+        <xdr:cNvPr id="11" name="/xl/media/image11.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra15624a87e004996"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc087f5aa59654a74"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -619,13 +654,13 @@
     <xdr:ext cx="10439400" cy="2076450"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="5f57e061-ded3-4082-9fa3-3887075b5eb1"/>
+        <xdr:cNvPr id="12" name="/xl/media/image12.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9ea7814966a4487d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2115ba9da17c4b47"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -646,13 +681,13 @@
     <xdr:ext cx="10439400" cy="1933575"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="bcf7bb3a-1d6f-4c7c-97c4-d99655a3a393"/>
+        <xdr:cNvPr id="13" name="/xl/media/image13.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R612decbfd7924c37"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R034c461ff03f4d99"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -673,13 +708,13 @@
     <xdr:ext cx="10477500" cy="6191250"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="409229f8-b634-48a1-be83-73d06245e0be"/>
+        <xdr:cNvPr id="14" name="/xl/media/image14.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R186a178ddb724e93"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R71da0c8b1193414d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -700,13 +735,13 @@
     <xdr:ext cx="9144000" cy="7239000"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="6a9c3e7c-4d97-4d6b-b745-57238a9334d9"/>
+        <xdr:cNvPr id="15" name="/xl/media/image15.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R21a2b257e9734831"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0a22d5f31f0448af"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -727,13 +762,40 @@
     <xdr:ext cx="10439400" cy="1933575"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="16" name="f933cb59-1699-4284-a35e-2dc415c5cf7e"/>
+        <xdr:cNvPr id="16" name="/xl/media/image16.jpg"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd49dd05eea5641ce"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3ff37b3b853641ad"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>472</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="7620000" cy="5810250"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="dcdf80f6-8795-4b73-b984-5c6906e71ea4"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R38a8c29770644cd2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1284,6 +1346,294 @@
         <x:v>Obrazová reference: S07, S10 (list Reference).</x:v>
       </x:c>
     </x:row>
+    <x:row r="17" ht="145" customHeight="1">
+      <x:c r="A17" s="30" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="str">
+        <x:v>Výchozí vypnutí</x:v>
+      </x:c>
+      <x:c r="C17" s="30" t="str">
+        <x:v>Čistá instalace / RPi a síťový dohled</x:v>
+      </x:c>
+      <x:c r="D17" s="30" t="str">
+        <x:v>Na instalaci rozšíření bez konfigurace: sudo consolepi-control syslog status; systemctl is-enabled consolepi-syslog. Zachytit provoz vůči kolektoru.</x:v>
+      </x:c>
+      <x:c r="E17" s="30" t="str">
+        <x:v>Odesílání vypnuto, cíl a vlastní CA prázdné, fronta 0, služba disabled; žádný syslog provoz.</x:v>
+      </x:c>
+      <x:c r="F17" s="30"/>
+      <x:c r="G17" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H17" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="145" customHeight="1">
+      <x:c r="A18" s="30" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="str">
+        <x:v>Severity 0 až 7</x:v>
+      </x:c>
+      <x:c r="C18" s="30" t="str">
+        <x:v>RPi a kolektor</x:v>
+      </x:c>
+      <x:c r="D18" s="30" t="str">
+        <x:v>Na testovacím kolektoru nastavit práh 4 a vyvolat logger -t consolepi -p authpriv.warning SYSLOG_ACCEPT_4 a -p authpriv.info SYSLOG_ACCEPT_6. Opakovat pro práh 6. Pro prahy 0 a 7 použít zprávy emerg a debug.</x:v>
+      </x:c>
+      <x:c r="E18" s="30" t="str">
+        <x:v>Práh 4 přijme warning, nikoli info; práh 6 obě. Práh 0 přijme jen emerg; 7 přijme i debug. Doložit severity a jedinečné značky v kolektoru.</x:v>
+      </x:c>
+      <x:c r="F18" s="30"/>
+      <x:c r="G18" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H18" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="145" customHeight="1">
+      <x:c r="A19" s="30" t="str">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="str">
+        <x:v>Povolené zdroje a údaje</x:v>
+      </x:c>
+      <x:c r="C19" s="30" t="str">
+        <x:v>RPi, web a kolektor</x:v>
+      </x:c>
+      <x:c r="D19" s="30" t="str">
+        <x:v>Vyvolat konzolovou relaci, úspěšné/neúspěšné SSH a webové přihlášení, nft-input-drop a chybu vybrané služby. Poslat neškodnou značku přes nepovolený tag a do testovacího sériového přepisu.</x:v>
+      </x:c>
+      <x:c r="E19" s="30" t="str">
+        <x:v>Povolené události se přenesou podle severity. Nepovolený tag a značka pouze v přepisu se nepřenesou. Webový audit obsahuje výsledek a IP, ne heslo ani formulář.</x:v>
+      </x:c>
+      <x:c r="F19" s="30"/>
+      <x:c r="G19" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H19" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="145" customHeight="1">
+      <x:c r="A20" s="30" t="str">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="str">
+        <x:v>TLS a identita serveru</x:v>
+      </x:c>
+      <x:c r="C20" s="30" t="str">
+        <x:v>RPi a testovací TLS kolektor</x:v>
+      </x:c>
+      <x:c r="D20" s="30" t="str">
+        <x:v>Ověřit platnou systémovou CA nebo interní PEM CA. Pak vyzkoušet nedůvěryhodnou CA a certifikát s chybným DNS/IP. Kontrolovat síťový záznam a stav fronty.</x:v>
+      </x:c>
+      <x:c r="E20" s="30" t="str">
+        <x:v>Platná identita se připojí; chybná CA nebo jméno/IP se odmítne. Zprávy čekají ve frontě a nedochází k automatickému přechodu na nešifrované TCP.</x:v>
+      </x:c>
+      <x:c r="F20" s="30"/>
+      <x:c r="G20" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H20" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="145" customHeight="1">
+      <x:c r="A21" s="30" t="str">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="str">
+        <x:v>Rámování a testovací zpráva</x:v>
+      </x:c>
+      <x:c r="C21" s="30" t="str">
+        <x:v>Web a kolektor</x:v>
+      </x:c>
+      <x:c r="D21" s="30" t="str">
+        <x:v>Pro TLS a výslovně nastavené TCP ověřit octet-counting rámování RFC 5425 a obsah RFC 5424. Odeslat test při severity 0, 4, 6 a 7. Porovnat UI s příjmem kolektoru.</x:v>
+      </x:c>
+      <x:c r="E21" s="30" t="str">
+        <x:v>Kolektor přijme SYSLOG_TEST version=1.9.1 na nastavené severity, facility authpriv. Web potvrzuje lokální zápis; příjem musí být doložen samostatně.</x:v>
+      </x:c>
+      <x:c r="F21" s="30"/>
+      <x:c r="G21" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H21" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="145" customHeight="1">
+      <x:c r="A22" s="30" t="str">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="str">
+        <x:v>Výpadek a restart služby</x:v>
+      </x:c>
+      <x:c r="C22" s="30" t="str">
+        <x:v>RPi a kolektor</x:v>
+      </x:c>
+      <x:c r="D22" s="30" t="str">
+        <x:v>Odpojit testovací kolektor, vytvořit označené události, kontrolovat status a funkčnost konzolové relace. Restartovat jen consolepi-syslog a obnovit spojení.</x:v>
+      </x:c>
+      <x:c r="E22" s="30" t="str">
+        <x:v>Fronta přežije restart, služba opakuje spojení po 10 s a konzole funguje během výpadku. Po obnově doložit příjem; vyhodnotit případné duplicity a ztráty.</x:v>
+      </x:c>
+      <x:c r="F22" s="30"/>
+      <x:c r="G22" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H22" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="145" customHeight="1">
+      <x:c r="A23" s="30" t="str">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="str">
+        <x:v>Limit fronty a oprávnění</x:v>
+      </x:c>
+      <x:c r="C23" s="30" t="str">
+        <x:v>Vyhrazené RPi</x:v>
+      </x:c>
+      <x:c r="D23" s="30" t="str">
+        <x:v>Při výpadku testovacího kolektoru vytvořit více než 2 000 označených událostí. Kontrolovat dropped/pending; stat -c "%a %U" /etc/consolepi/syslog.json /var/lib/consolepi-syslog /var/lib/consolepi-syslog/queue.sqlite3.</x:v>
+      </x:c>
+      <x:c r="E23" s="30" t="str">
+        <x:v>Nejvýše 2 000 zpráv, nejstarší se zahodí a dropped vzroste. Konfigurace a DB 0600, adresář 0700, vlastník root.</x:v>
+      </x:c>
+      <x:c r="F23" s="30"/>
+      <x:c r="G23" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H23" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="145" customHeight="1">
+      <x:c r="A24" s="30" t="str">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="str">
+        <x:v>Změna cíle a vypnutí</x:v>
+      </x:c>
+      <x:c r="C24" s="30" t="str">
+        <x:v>Vyhrazené RPi a dva kolektory</x:v>
+      </x:c>
+      <x:c r="D24" s="30" t="str">
+        <x:v>Vytvořit čekající události při výpadku. Uložit jiný cíl a ověřit oba kolektory. Samostatně opakovat změnu severity a vypnutí.</x:v>
+      </x:c>
+      <x:c r="E24" s="30" t="str">
+        <x:v>Každé uložení a vypnutí vyprázdní frontu. Staré zprávy nedorazí na nový cíl. Nově vzniklé povolené zprávy se řídí novou konfigurací.</x:v>
+      </x:c>
+      <x:c r="F24" s="30"/>
+      <x:c r="G24" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H24" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="145" customHeight="1">
+      <x:c r="A25" s="30" t="str">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="str">
+        <x:v>Ochrana webového nastavení</x:v>
+      </x:c>
+      <x:c r="C25" s="30" t="str">
+        <x:v>Prohlížeč / testovací klient</x:v>
+      </x:c>
+      <x:c r="D25" s="30" t="str">
+        <x:v>Zkusit POST /system/syslog bez přihlášení, bez/nesprávného CSRF, s nepovolenou akcí, neplatným portem, severity a CA. S přihlášením a správným tokenem uložit platné nastavení.</x:v>
+      </x:c>
+      <x:c r="E25" s="30" t="str">
+        <x:v>Neoprávněné nebo neplatné požadavky nezmění nastavení. Platný požadavek je přijat. Při selhání aktivace se obnoví předchozí konfigurace.</x:v>
+      </x:c>
+      <x:c r="F25" s="30"/>
+      <x:c r="G25" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H25" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="145" customHeight="1">
+      <x:c r="A26" s="30" t="str">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="str">
+        <x:v>Reset a sanitizace image</x:v>
+      </x:c>
+      <x:c r="C26" s="30" t="str">
+        <x:v>Vyhrazené testovací médium</x:v>
+      </x:c>
+      <x:c r="D26" s="30" t="str">
+        <x:v>Po záloze a se souhlasem vlastníka testovacího zařízení nastavit cíl, CA a frontu. Samostatně ověřit tovární reset a postup generic image včetně validátoru.</x:v>
+      </x:c>
+      <x:c r="E26" s="30" t="str">
+        <x:v>Cíl a vlastní CA odstraněny, fronta prázdná, syslog vypnutý a služba disabled. Validátor potvrdí čistý stav.</x:v>
+      </x:c>
+      <x:c r="F26" s="30"/>
+      <x:c r="G26" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H26" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="145" customHeight="1">
+      <x:c r="A27" s="30" t="str">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="str">
+        <x:v>Záloha a obnova</x:v>
+      </x:c>
+      <x:c r="C27" s="30" t="str">
+        <x:v>Vyhrazené testovací RPi</x:v>
+      </x:c>
+      <x:c r="D27" s="30" t="str">
+        <x:v>Se zapnutým syslogem a frontou vytvořit šifrovanou zálohu. Obnovit ji na testovacím zařízení. Kontrolovat konfiguraci, validaci a nepřenesení starých čekajících událostí.</x:v>
+      </x:c>
+      <x:c r="E27" s="30" t="str">
+        <x:v>Záloha obsahuje konfiguraci, nikoli frontu. Obnova validuje konfiguraci před aktivací; čekající zprávy z původního zařízení se neobnoví.</x:v>
+      </x:c>
+      <x:c r="F27" s="30"/>
+      <x:c r="G27" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H27" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="145" customHeight="1">
+      <x:c r="A28" s="30" t="str">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B28" s="30" t="str">
+        <x:v>Důkaz nasazené verze</x:v>
+      </x:c>
+      <x:c r="C28" s="30" t="str">
+        <x:v>RPi a distribuční soubory</x:v>
+      </x:c>
+      <x:c r="D28" s="30" t="str">
+        <x:v>Zaznamenat VERSION, commit/identifikaci nasazeného balíčku, SHA-256 balíčku a přítomnost syslog služby. Porovnat se zdroji PR 22 a s původním vydáním 2. 10. 2026.</x:v>
+      </x:c>
+      <x:c r="E28" s="30" t="str">
+        <x:v>Důkaz rozlišuje zdrojové rozšíření od původního image 1.9.1 bez syslogu. VERSION samotná nestačí; příjem v kolektoru je doložen zvlášť.</x:v>
+      </x:c>
+      <x:c r="F28" s="30"/>
+      <x:c r="G28" s="30" t="str">
+        <x:v>☐ Nevyhodnoceno</x:v>
+      </x:c>
+      <x:c r="H28" s="30" t="str">
+        <x:v>Syslog zdrojové rozšíření PR 22; S17 je lokální náhled. Doplnit skutečný důkaz z RPi a kolektoru.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -1300,8 +1650,22 @@
       <x:formula>G7="— N/A"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:conditionalFormatting sqref="G17:G28">
+    <x:cfRule type="expression" dxfId="6" priority="4">
+      <x:formula>G17="☑ Akceptováno"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="7" priority="5">
+      <x:formula>G17="☒ Neakceptováno"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="8" priority="6">
+      <x:formula>G17="— N/A"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="G7:G16">
+      <x:formula1>"☐ Nevyhodnoceno,☑ Akceptováno,☒ Neakceptováno,— N/A"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G17:G28">
       <x:formula1>"☐ Nevyhodnoceno,☑ Akceptováno,☒ Neakceptováno,— N/A"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -1348,8 +1712,8 @@
         <x:v>Celkem testů</x:v>
       </x:c>
       <x:c r="B4" s="29" t="n">
-        <x:f>COUNTA('Akceptační testy'!A7:A16)</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTA('Akceptační testy'!A7:A28)</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C4" s="29"/>
       <x:c r="D4" s="29"/>
@@ -1359,7 +1723,7 @@
         <x:v>Akceptováno</x:v>
       </x:c>
       <x:c r="B5" s="29" t="n">
-        <x:f>COUNTIF('Akceptační testy'!G7:G16,"☑ Akceptováno")</x:f>
+        <x:f>COUNTIF('Akceptační testy'!G7:G28,"☑ Akceptováno")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="29"/>
@@ -1370,7 +1734,7 @@
         <x:v>Neakceptováno</x:v>
       </x:c>
       <x:c r="B6" s="29" t="n">
-        <x:f>COUNTIF('Akceptační testy'!G7:G16,"☒ Neakceptováno")</x:f>
+        <x:f>COUNTIF('Akceptační testy'!G7:G28,"☒ Neakceptováno")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="29"/>
@@ -1381,7 +1745,7 @@
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="B7" s="29" t="n">
-        <x:f>COUNTIF('Akceptační testy'!G7:G16,"— N/A")</x:f>
+        <x:f>COUNTIF('Akceptační testy'!G7:G28,"— N/A")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="29"/>
@@ -1392,8 +1756,8 @@
         <x:v>Nevyhodnoceno</x:v>
       </x:c>
       <x:c r="B8" s="29" t="n">
-        <x:f>COUNTIF('Akceptační testy'!G7:G16,"☐ Nevyhodnoceno")</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTIF('Akceptační testy'!G7:G28,"☐ Nevyhodnoceno")</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C8" s="29"/>
       <x:c r="D8" s="29"/>
@@ -2276,6 +2640,107 @@
     <x:row r="443" ht="15" customHeight="1"/>
     <x:row r="444" ht="15" customHeight="1"/>
     <x:row r="445" ht="15" customHeight="1"/>
+    <x:row r="460" ht="26" customHeight="1">
+      <x:c r="A460" s="59" t="str">
+        <x:v>Syslog rozšíření zdrojů 1.9.1 doplněno 8. 10. 2026</x:v>
+      </x:c>
+      <x:c r="B460" s="59"/>
+      <x:c r="C460" s="59"/>
+    </x:row>
+    <x:row r="461" ht="24" customHeight="1">
+      <x:c r="A461" s="61" t="str">
+        <x:v>S17 je lokální náhled šablony, nikoli snímek nasazené funkce na RPi. Původní image a archivy z 2. 10. 2026 syslog neobsahují. Místně prošlo 14 kontrol backendu a 6 kontrol webu; akceptační testy 11–22 zůstávají Nevyhodnoceno.</x:v>
+      </x:c>
+      <x:c r="B461" s="61"/>
+      <x:c r="C461" s="61"/>
+    </x:row>
+    <x:row r="462" ht="24" customHeight="1">
+      <x:c r="A462" s="61"/>
+      <x:c r="B462" s="61"/>
+      <x:c r="C462" s="61"/>
+    </x:row>
+    <x:row r="463" ht="24" customHeight="1">
+      <x:c r="A463" s="61"/>
+      <x:c r="B463" s="61"/>
+      <x:c r="C463" s="61"/>
+    </x:row>
+    <x:row r="465" ht="45" customHeight="1">
+      <x:c r="A465" s="61" t="str">
+        <x:v>Specifikace</x:v>
+      </x:c>
+      <x:c r="B465" s="61" t="str">
+        <x:v>Vzdálený syslog</x:v>
+      </x:c>
+      <x:c r="C465" s="61" t="str">
+        <x:v>https://github.com/jiriflos-eng/ConsolePi-Plus/blob/codex/syslog-1.9.1/docs/SYSLOG.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="466" ht="45" customHeight="1">
+      <x:c r="A466" s="61" t="str">
+        <x:v>Implementace a ověření</x:v>
+      </x:c>
+      <x:c r="B466" s="61" t="str">
+        <x:v>PR 22</x:v>
+      </x:c>
+      <x:c r="C466" s="61" t="str">
+        <x:v>https://github.com/jiriflos-eng/ConsolePi-Plus/pull/22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="468" ht="26" customHeight="1">
+      <x:c r="A468" s="59" t="str">
+        <x:v>S17 Nastavení vzdáleného syslogu</x:v>
+      </x:c>
+      <x:c r="B468" s="59"/>
+      <x:c r="C468" s="59"/>
+    </x:row>
+    <x:row r="469" ht="24" customHeight="1">
+      <x:c r="A469" s="61" t="str">
+        <x:v>Lokální náhled z 8. 10. 2026: vypnuto, TCP/TLS, port 6514, práh 6, veřejná CA a fronta. Zdroj: šablona system.html, PR 22. Obrázek slouží k orientaci; nedokládá doručení ani akceptaci.</x:v>
+      </x:c>
+      <x:c r="B469" s="61"/>
+      <x:c r="C469" s="61"/>
+    </x:row>
+    <x:row r="470" ht="24" customHeight="1">
+      <x:c r="A470" s="61"/>
+      <x:c r="B470" s="61"/>
+      <x:c r="C470" s="61"/>
+    </x:row>
+    <x:row r="471" ht="24" customHeight="1">
+      <x:c r="A471" s="61"/>
+      <x:c r="B471" s="61"/>
+      <x:c r="C471" s="61"/>
+    </x:row>
+    <x:row r="473" ht="15" customHeight="1"/>
+    <x:row r="474" ht="15" customHeight="1"/>
+    <x:row r="475" ht="15" customHeight="1"/>
+    <x:row r="476" ht="15" customHeight="1"/>
+    <x:row r="477" ht="15" customHeight="1"/>
+    <x:row r="478" ht="15" customHeight="1"/>
+    <x:row r="479" ht="15" customHeight="1"/>
+    <x:row r="480" ht="15" customHeight="1"/>
+    <x:row r="481" ht="15" customHeight="1"/>
+    <x:row r="482" ht="15" customHeight="1"/>
+    <x:row r="483" ht="15" customHeight="1"/>
+    <x:row r="484" ht="15" customHeight="1"/>
+    <x:row r="485" ht="15" customHeight="1"/>
+    <x:row r="486" ht="15" customHeight="1"/>
+    <x:row r="487" ht="15" customHeight="1"/>
+    <x:row r="488" ht="15" customHeight="1"/>
+    <x:row r="489" ht="15" customHeight="1"/>
+    <x:row r="490" ht="15" customHeight="1"/>
+    <x:row r="491" ht="15" customHeight="1"/>
+    <x:row r="492" ht="15" customHeight="1"/>
+    <x:row r="493" ht="15" customHeight="1"/>
+    <x:row r="494" ht="15" customHeight="1"/>
+    <x:row r="495" ht="15" customHeight="1"/>
+    <x:row r="496" ht="15" customHeight="1"/>
+    <x:row r="497" ht="15" customHeight="1"/>
+    <x:row r="498" ht="15" customHeight="1"/>
+    <x:row r="499" ht="15" customHeight="1"/>
+    <x:row r="500" ht="15" customHeight="1"/>
+    <x:row r="501" ht="15" customHeight="1"/>
+    <x:row r="502" ht="15" customHeight="1"/>
+    <x:row r="503" ht="15" customHeight="1"/>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:C1"/>
@@ -2314,8 +2779,12 @@
     <x:mergeCell ref="A388:C389"/>
     <x:mergeCell ref="A431:C431"/>
     <x:mergeCell ref="A432:C433"/>
+    <x:mergeCell ref="A460:C460"/>
+    <x:mergeCell ref="A461:C463"/>
+    <x:mergeCell ref="A468:C468"/>
+    <x:mergeCell ref="A469:C471"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77a66083822b42dc"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45a2b7d2b6e444af"/>
 </x:worksheet>
 </file>
</xml_diff>